<commit_message>
Mejorar la comunicación visual de los boletines
Recupera la identidad visual institucional de En proceso, Suficiente y Avanzado, diferencia dato, vacío y período futuro, y neutraliza la plantilla base.

La lógica queda centralizada para informes individuales y por curso, con filas dinámicas y 225/225 tests OK.
</commit_message>
<xml_diff>
--- a/src/Generador_EPS_v0_4.xlsx
+++ b/src/Generador_EPS_v0_4.xlsx
@@ -1021,13 +1021,13 @@
       </x:c>
       <x:c r="D9" s="31"/>
       <x:c r="E9" s="19"/>
-      <x:c r="F9" s="20"/>
+      <x:c r="F9" s="19"/>
       <x:c r="G9" s="19"/>
-      <x:c r="H9" s="20"/>
-      <x:c r="I9" s="20"/>
-      <x:c r="J9" s="20"/>
-      <x:c r="K9" s="20"/>
-      <x:c r="L9" s="20"/>
+      <x:c r="H9" s="19"/>
+      <x:c r="I9" s="19"/>
+      <x:c r="J9" s="19"/>
+      <x:c r="K9" s="19"/>
+      <x:c r="L9" s="19"/>
       <x:c r="M9" s="21"/>
     </x:row>
     <x:row r="10" ht="35.25" customHeight="1">
@@ -1037,13 +1037,13 @@
       </x:c>
       <x:c r="D10" s="31"/>
       <x:c r="E10" s="19"/>
-      <x:c r="F10" s="20"/>
+      <x:c r="F10" s="19"/>
       <x:c r="G10" s="19"/>
-      <x:c r="H10" s="20"/>
-      <x:c r="I10" s="20"/>
-      <x:c r="J10" s="20"/>
-      <x:c r="K10" s="20"/>
-      <x:c r="L10" s="20"/>
+      <x:c r="H10" s="19"/>
+      <x:c r="I10" s="19"/>
+      <x:c r="J10" s="19"/>
+      <x:c r="K10" s="19"/>
+      <x:c r="L10" s="19"/>
       <x:c r="M10" s="21"/>
     </x:row>
     <x:row r="11" ht="35.25" customHeight="1">
@@ -1053,13 +1053,13 @@
       </x:c>
       <x:c r="D11" s="31"/>
       <x:c r="E11" s="19"/>
-      <x:c r="F11" s="20"/>
+      <x:c r="F11" s="19"/>
       <x:c r="G11" s="19"/>
-      <x:c r="H11" s="20"/>
-      <x:c r="I11" s="20"/>
-      <x:c r="J11" s="20"/>
-      <x:c r="K11" s="20"/>
-      <x:c r="L11" s="20"/>
+      <x:c r="H11" s="19"/>
+      <x:c r="I11" s="19"/>
+      <x:c r="J11" s="19"/>
+      <x:c r="K11" s="19"/>
+      <x:c r="L11" s="19"/>
       <x:c r="M11" s="21"/>
     </x:row>
     <x:row r="12" ht="35.25" customHeight="1">
@@ -1069,13 +1069,13 @@
       </x:c>
       <x:c r="D12" s="31"/>
       <x:c r="E12" s="19"/>
-      <x:c r="F12" s="20"/>
+      <x:c r="F12" s="19"/>
       <x:c r="G12" s="19"/>
-      <x:c r="H12" s="20"/>
-      <x:c r="I12" s="20"/>
-      <x:c r="J12" s="20"/>
-      <x:c r="K12" s="20"/>
-      <x:c r="L12" s="20"/>
+      <x:c r="H12" s="19"/>
+      <x:c r="I12" s="19"/>
+      <x:c r="J12" s="19"/>
+      <x:c r="K12" s="19"/>
+      <x:c r="L12" s="19"/>
       <x:c r="M12" s="21"/>
     </x:row>
     <x:row r="13" ht="35.25" customHeight="1">
@@ -1085,13 +1085,13 @@
       </x:c>
       <x:c r="D13" s="31"/>
       <x:c r="E13" s="19"/>
-      <x:c r="F13" s="20"/>
+      <x:c r="F13" s="19"/>
       <x:c r="G13" s="19"/>
-      <x:c r="H13" s="20"/>
-      <x:c r="I13" s="20"/>
-      <x:c r="J13" s="20"/>
-      <x:c r="K13" s="20"/>
-      <x:c r="L13" s="20"/>
+      <x:c r="H13" s="19"/>
+      <x:c r="I13" s="19"/>
+      <x:c r="J13" s="19"/>
+      <x:c r="K13" s="19"/>
+      <x:c r="L13" s="19"/>
       <x:c r="M13" s="21"/>
     </x:row>
     <x:row r="14" ht="35.25" customHeight="1">
@@ -1101,13 +1101,13 @@
       </x:c>
       <x:c r="D14" s="31"/>
       <x:c r="E14" s="19"/>
-      <x:c r="F14" s="20"/>
+      <x:c r="F14" s="19"/>
       <x:c r="G14" s="19"/>
-      <x:c r="H14" s="20"/>
-      <x:c r="I14" s="20"/>
-      <x:c r="J14" s="20"/>
-      <x:c r="K14" s="20"/>
-      <x:c r="L14" s="20"/>
+      <x:c r="H14" s="19"/>
+      <x:c r="I14" s="19"/>
+      <x:c r="J14" s="19"/>
+      <x:c r="K14" s="19"/>
+      <x:c r="L14" s="19"/>
       <x:c r="M14" s="21"/>
     </x:row>
     <x:row r="15" ht="35.25" customHeight="1">
@@ -1117,13 +1117,13 @@
       </x:c>
       <x:c r="D15" s="31"/>
       <x:c r="E15" s="19"/>
-      <x:c r="F15" s="20"/>
+      <x:c r="F15" s="19"/>
       <x:c r="G15" s="19"/>
-      <x:c r="H15" s="20"/>
-      <x:c r="I15" s="20"/>
-      <x:c r="J15" s="20"/>
-      <x:c r="K15" s="20"/>
-      <x:c r="L15" s="20"/>
+      <x:c r="H15" s="19"/>
+      <x:c r="I15" s="19"/>
+      <x:c r="J15" s="19"/>
+      <x:c r="K15" s="19"/>
+      <x:c r="L15" s="19"/>
       <x:c r="M15" s="21"/>
     </x:row>
     <x:row r="16" ht="38.25" customHeight="1">
@@ -1133,13 +1133,13 @@
       </x:c>
       <x:c r="D16" s="31"/>
       <x:c r="E16" s="19"/>
-      <x:c r="F16" s="20"/>
+      <x:c r="F16" s="19"/>
       <x:c r="G16" s="19"/>
-      <x:c r="H16" s="20"/>
-      <x:c r="I16" s="20"/>
-      <x:c r="J16" s="20"/>
-      <x:c r="K16" s="20"/>
-      <x:c r="L16" s="20"/>
+      <x:c r="H16" s="19"/>
+      <x:c r="I16" s="19"/>
+      <x:c r="J16" s="19"/>
+      <x:c r="K16" s="19"/>
+      <x:c r="L16" s="19"/>
       <x:c r="M16" s="21"/>
     </x:row>
     <x:row r="17" ht="192" customHeight="1">
@@ -14915,28 +14915,6 @@
     <x:mergeCell ref="E4:F4"/>
     <x:mergeCell ref="E5:F5"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E9:E16">
-    <x:cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
-      <x:formula>"En Proceso"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <x:formula>"Suficiente"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
-      <x:formula>"Avanzado"</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G9:G16">
-    <x:cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <x:formula>"En Proceso"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
-      <x:formula>"Suficiente"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
-      <x:formula>"Avanzado"</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1e090b917046da"/>
 </x:worksheet>

</xml_diff>